<commit_message>
Populate Calves/Steers avg price from herdsman's Animal Scenarios & Costs data
</commit_message>
<xml_diff>
--- a/data/Annual Summary by Category.xlsx
+++ b/data/Annual Summary by Category.xlsx
@@ -460,6 +460,9 @@
           <t>Calves</t>
         </is>
       </c>
+      <c r="C2" t="n">
+        <v>1500</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -473,6 +476,9 @@
         <is>
           <t>Steers</t>
         </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3500</v>
       </c>
     </row>
     <row r="5">

</xml_diff>